<commit_message>
Western re-measurement with fixed AM Best parsers — +44 upgrades 0 downgrades (UT +20: 57% of blocks were header-dropped; NM +14, NV +5, AZ +4, MT +1); 432 cross-checked (332 direct); NM artifacts force-added (gitignore gap); 0 rate-cell changes
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Insurance Rate Data Scraper/output/az_final_rates.xlsx
+++ b/Insurance Rate Data Scraper/output/az_final_rates.xlsx
@@ -1710,7 +1710,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>pipeline_only</t>
+          <t>ambest_validated</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1720,10 +1720,14 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>pipeline_extracted_in_validated_window</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>ambest_cross_checked</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -15021,7 +15025,7 @@
       </c>
       <c r="R145" t="inlineStr">
         <is>
-          <t>pipeline_only</t>
+          <t>ambest_validated</t>
         </is>
       </c>
       <c r="S145" t="inlineStr">
@@ -15031,10 +15035,14 @@
       </c>
       <c r="T145" t="inlineStr">
         <is>
-          <t>pipeline_extracted_in_validated_window</t>
-        </is>
-      </c>
-      <c r="U145" t="inlineStr"/>
+          <t>ambest_cross_checked</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -15117,7 +15125,7 @@
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>pipeline_only</t>
+          <t>ambest_validated</t>
         </is>
       </c>
       <c r="S146" t="inlineStr">
@@ -15127,10 +15135,14 @@
       </c>
       <c r="T146" t="inlineStr">
         <is>
-          <t>pipeline_extracted_in_validated_window</t>
-        </is>
-      </c>
-      <c r="U146" t="inlineStr"/>
+          <t>ambest_cross_checked</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -17955,7 +17967,7 @@
       </c>
       <c r="R174" t="inlineStr">
         <is>
-          <t>pipeline_only</t>
+          <t>ambest_validated</t>
         </is>
       </c>
       <c r="S174" t="inlineStr">
@@ -17965,10 +17977,14 @@
       </c>
       <c r="T174" t="inlineStr">
         <is>
-          <t>pipeline_extracted_in_validated_window</t>
-        </is>
-      </c>
-      <c r="U174" t="inlineStr"/>
+          <t>ambest_cross_checked</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">

</xml_diff>

<commit_message>
3rd AM Best block-extraction fix (blank max%/min% + non-ASCII minus normalization, same family as 0362b02 / aa4fe36); +12 genuine direct matches (AZ +2, GA +10), recovers SFMA-134114404 the 1.2M-ph false negative; label-only, 0 rate-cell changes, anchor 14/14
Backlog B1 (consolidate 6 AM Best parsers into one blank-safe extractor) + separate-issue notes B2 (UT date-column), B3 (GA/HO Safeco value discrepancy - possible deliverable concern), B4 (NV Progressive genuine absence). Harness scripts committed prior in d15577f.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Insurance Rate Data Scraper/output/az_final_rates.xlsx
+++ b/Insurance Rate Data Scraper/output/az_final_rates.xlsx
@@ -15220,7 +15220,7 @@
       </c>
       <c r="R147" t="inlineStr">
         <is>
-          <t>pipeline_only</t>
+          <t>ambest_validated</t>
         </is>
       </c>
       <c r="S147" t="inlineStr">
@@ -15230,10 +15230,14 @@
       </c>
       <c r="T147" t="inlineStr">
         <is>
-          <t>pipeline_extracted_in_validated_window</t>
-        </is>
-      </c>
-      <c r="U147" t="inlineStr"/>
+          <t>ambest_cross_checked</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -15311,7 +15315,7 @@
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>pipeline_only</t>
+          <t>ambest_validated</t>
         </is>
       </c>
       <c r="S148" t="inlineStr">
@@ -15321,10 +15325,14 @@
       </c>
       <c r="T148" t="inlineStr">
         <is>
-          <t>pipeline_extracted_in_validated_window</t>
-        </is>
-      </c>
-      <c r="U148" t="inlineStr"/>
+          <t>ambest_cross_checked</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">

</xml_diff>